<commit_message>
fin de la practica 3 y por poco de mi vida :(((
</commit_message>
<xml_diff>
--- a/resources/SistemasBasura.xlsx
+++ b/resources/SistemasBasura.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1269" uniqueCount="667">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1314" uniqueCount="710">
   <si>
     <t>Nombre</t>
   </si>
@@ -1576,12 +1576,24 @@
     <t>3162456104254692000A</t>
   </si>
   <si>
+    <t>31645124453461205100</t>
+  </si>
+  <si>
+    <t>65614874115615445600</t>
+  </si>
+  <si>
+    <t>32569523086220165100</t>
+  </si>
+  <si>
     <t>MC6436520125638451012515</t>
   </si>
   <si>
     <t>rgo00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>21584976912154655485</t>
+  </si>
+  <si>
     <t>ES9621584976912154655485</t>
   </si>
   <si>
@@ -1600,12 +1612,18 @@
     <t>abp00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>21564975263245467900</t>
+  </si>
+  <si>
     <t>LT2132566221532587754888</t>
   </si>
   <si>
     <t>acp00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>00750184350702510003</t>
+  </si>
+  <si>
     <t>74635623W</t>
   </si>
   <si>
@@ -1627,6 +1645,9 @@
     <t>83647564Z</t>
   </si>
   <si>
+    <t>25030000194574745400</t>
+  </si>
+  <si>
     <t>AT7125030000194574745400</t>
   </si>
   <si>
@@ -1645,6 +1666,9 @@
     <t>92736981S</t>
   </si>
   <si>
+    <t>20960043033096200013</t>
+  </si>
+  <si>
     <t>ES6520960043033096200013</t>
   </si>
   <si>
@@ -1669,6 +1693,9 @@
     <t>pp00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>12669681125112121200</t>
+  </si>
+  <si>
     <t>DE6912669681125112121200</t>
   </si>
   <si>
@@ -1687,6 +1714,9 @@
     <t>cgm00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>64578946720051516403</t>
+  </si>
+  <si>
     <t>ES4534698752714600549403</t>
   </si>
   <si>
@@ -1696,6 +1726,9 @@
     <t>25147854E</t>
   </si>
   <si>
+    <t>23185484415641685908</t>
+  </si>
+  <si>
     <t>FR8423185484415641685908</t>
   </si>
   <si>
@@ -1735,6 +1768,9 @@
     <t>dlr00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>75647586157564758698</t>
+  </si>
+  <si>
     <t>FI6775647586157564758698</t>
   </si>
   <si>
@@ -1783,24 +1819,39 @@
     <t>iag00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>25635478301002541233</t>
+  </si>
+  <si>
     <t>SM7825635478301002541233</t>
   </si>
   <si>
     <t>gpg00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>32154697155423121012</t>
+  </si>
+  <si>
     <t>ES8932154697155423121012</t>
   </si>
   <si>
     <t>rgg00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>20008521588775113327</t>
+  </si>
+  <si>
     <t>GB5720008521588775113327</t>
   </si>
   <si>
     <t>afg00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>20960043073000100018</t>
+  </si>
+  <si>
+    <t>12548523445214585218</t>
+  </si>
+  <si>
     <t>ES0912548523445214585218</t>
   </si>
   <si>
@@ -1819,6 +1870,9 @@
     <t>lr00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>20960031482124800018</t>
+  </si>
+  <si>
     <t>ES2420960031482124800018</t>
   </si>
   <si>
@@ -1843,12 +1897,18 @@
     <t>rog00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>20960043023000100021</t>
+  </si>
+  <si>
     <t>ES6020960043023000100021</t>
   </si>
   <si>
     <t>sog00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>65168874681561561522</t>
+  </si>
+  <si>
     <t>ES2965168874681561561522</t>
   </si>
   <si>
@@ -1861,6 +1921,9 @@
     <t>mbg00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>21416325801510005527</t>
+  </si>
+  <si>
     <t>ES7421416325801510005527</t>
   </si>
   <si>
@@ -1879,18 +1942,27 @@
     <t>12345679S</t>
   </si>
   <si>
+    <t>20960056143231500032</t>
+  </si>
+  <si>
     <t>ES6620960056143231500032</t>
   </si>
   <si>
     <t>fdl00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>63516541858944000993</t>
+  </si>
+  <si>
     <t>ES4063516541858944000993</t>
   </si>
   <si>
     <t>sdm00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>23658965294585223213</t>
+  </si>
+  <si>
     <t>ES2923658965294585223213</t>
   </si>
   <si>
@@ -1903,12 +1975,18 @@
     <t>gpm00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>23652365132254222021</t>
+  </si>
+  <si>
     <t>ES5223652365132254222021</t>
   </si>
   <si>
     <t>eam00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>20012541120023365296</t>
+  </si>
+  <si>
     <t>ES9232584216971684051000</t>
   </si>
   <si>
@@ -1927,12 +2005,18 @@
     <t>bdc00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>36245978123245679018</t>
+  </si>
+  <si>
     <t>ES4836245978123245679018</t>
   </si>
   <si>
     <t>ngc00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>87635467511625345671</t>
+  </si>
+  <si>
     <t>ES2987635467511625345671</t>
   </si>
   <si>
@@ -1945,24 +2029,36 @@
     <t>mlc01@tasabasura2026.com</t>
   </si>
   <si>
+    <t>20960043093468900021</t>
+  </si>
+  <si>
     <t>ES4820960043093468900021</t>
   </si>
   <si>
     <t>cfc00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>84729478014857627845</t>
+  </si>
+  <si>
     <t>ES7884729478014857627845</t>
   </si>
   <si>
     <t>cgc00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>85550564796165145618</t>
+  </si>
+  <si>
     <t>ES1665165654918886005001</t>
   </si>
   <si>
     <t>ksc00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>65645150815168448846</t>
+  </si>
+  <si>
     <t>AT9465645150815168448846</t>
   </si>
   <si>
@@ -1981,46 +2077,79 @@
     <t>mfd00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>51556584261251000242</t>
+  </si>
+  <si>
     <t>IE4751556584261251000242</t>
   </si>
   <si>
     <t>gmm02@tasabasura2026.com</t>
   </si>
   <si>
+    <t>87457619137384957654</t>
+  </si>
+  <si>
+    <t>87457619164384957654</t>
+  </si>
+  <si>
     <t>LT1687457619164384957654</t>
   </si>
   <si>
     <t>dmc00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>87457619177384957657</t>
+  </si>
+  <si>
     <t>ES9587457619177384957657</t>
   </si>
   <si>
     <t>ebc00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>87457619117384957658</t>
+  </si>
+  <si>
+    <t>87457619167384957659</t>
+  </si>
+  <si>
     <t>ES0687457619167384957659</t>
   </si>
   <si>
     <t>msc00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>87457619117384957651</t>
+  </si>
+  <si>
     <t>ES4787457619117384957651</t>
   </si>
   <si>
     <t>mdc00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>87457619197384957653</t>
+  </si>
+  <si>
     <t>ES7987457619197384957653</t>
   </si>
   <si>
     <t>mfc00@tasabasura2026.com</t>
   </si>
   <si>
+    <t>87457619187384957617</t>
+  </si>
+  <si>
     <t>ES4687457619187384957617</t>
   </si>
   <si>
     <t>cdd00@tasabasura2026.com</t>
+  </si>
+  <si>
+    <t>87457619177384957619</t>
+  </si>
+  <si>
+    <t>87457619187384957621</t>
   </si>
   <si>
     <t>AT6887457619187384957621</t>
@@ -2485,7 +2614,7 @@
         <v>476</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>444</v>
+        <v>516</v>
       </c>
       <c r="K2" t="s" s="0">
         <v>232</v>
@@ -2529,7 +2658,7 @@
         <v>477</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>445</v>
+        <v>517</v>
       </c>
       <c r="K3" t="s" s="0">
         <v>232</v>
@@ -2571,7 +2700,7 @@
         <v>478</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>446</v>
+        <v>518</v>
       </c>
       <c r="K4" t="s" s="0">
         <v>232</v>
@@ -2662,10 +2791,10 @@
         <v>235</v>
       </c>
       <c r="I6" t="s" s="0">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="J6" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="K6" t="s">
         <v>232</v>
@@ -2709,13 +2838,13 @@
         <v>438</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>507</v>
+        <v>521</v>
       </c>
       <c r="I7" t="s" s="0">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="J7" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="K7" t="s">
         <v>232</v>
@@ -2762,10 +2891,10 @@
         <v>236</v>
       </c>
       <c r="I8" t="s" s="0">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="J8" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="K8" t="s">
         <v>232</v>
@@ -2856,10 +2985,10 @@
         <v>238</v>
       </c>
       <c r="I10" t="s" s="0">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="J10" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="K10" t="s">
         <v>232</v>
@@ -2903,7 +3032,7 @@
         <v>481</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>447</v>
+        <v>528</v>
       </c>
       <c r="K11" t="s" s="0">
         <v>232</v>
@@ -2950,10 +3079,10 @@
         <v>411</v>
       </c>
       <c r="I12" t="s" s="0">
-        <v>524</v>
+        <v>529</v>
       </c>
       <c r="J12" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
       <c r="K12" t="s">
         <v>232</v>
@@ -3039,7 +3168,7 @@
         <v>410</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>509</v>
+        <v>531</v>
       </c>
       <c r="K14" t="s" s="0">
         <v>232</v>
@@ -3084,16 +3213,16 @@
         <v>141</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>412</v>
       </c>
       <c r="I16" t="s" s="0">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="J16" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="K16" t="s">
         <v>232</v>
@@ -3132,16 +3261,16 @@
         <v>141</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>413</v>
       </c>
       <c r="I17" t="s" s="0">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="J17" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="K17" t="s">
         <v>232</v>
@@ -3180,16 +3309,16 @@
         <v>142</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>448</v>
+        <v>539</v>
       </c>
       <c r="I18" t="s" s="0">
-        <v>533</v>
+        <v>540</v>
       </c>
       <c r="J18" t="s">
-        <v>534</v>
+        <v>541</v>
       </c>
       <c r="K18" t="s">
         <v>232</v>
@@ -3228,16 +3357,16 @@
         <v>142</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>414</v>
       </c>
       <c r="I19" t="s" s="0">
-        <v>536</v>
+        <v>543</v>
       </c>
       <c r="J19" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
       <c r="K19" t="s">
         <v>232</v>
@@ -3276,16 +3405,16 @@
         <v>143</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>538</v>
+        <v>545</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>508</v>
+        <v>546</v>
       </c>
       <c r="I20" t="s" s="0">
-        <v>539</v>
+        <v>547</v>
       </c>
       <c r="J20" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="K20" t="s">
         <v>232</v>
@@ -3369,10 +3498,10 @@
         <v>416</v>
       </c>
       <c r="I22" t="s" s="0">
-        <v>541</v>
+        <v>549</v>
       </c>
       <c r="J22" t="s">
-        <v>542</v>
+        <v>550</v>
       </c>
       <c r="K22" t="s">
         <v>232</v>
@@ -3411,13 +3540,13 @@
         <v>172</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>449</v>
+        <v>239</v>
       </c>
       <c r="I23" t="s" s="0">
-        <v>543</v>
+        <v>551</v>
       </c>
       <c r="J23" t="s">
-        <v>544</v>
+        <v>552</v>
       </c>
       <c r="K23" t="s">
         <v>232</v>
@@ -3459,10 +3588,10 @@
         <v>417</v>
       </c>
       <c r="I24" t="s" s="0">
-        <v>545</v>
+        <v>553</v>
       </c>
       <c r="J24" t="s">
-        <v>546</v>
+        <v>554</v>
       </c>
       <c r="K24" t="s">
         <v>232</v>
@@ -3501,13 +3630,13 @@
         <v>174</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>450</v>
+        <v>555</v>
       </c>
       <c r="I25" t="s" s="0">
-        <v>547</v>
+        <v>556</v>
       </c>
       <c r="J25" t="s">
-        <v>548</v>
+        <v>557</v>
       </c>
       <c r="K25" t="s">
         <v>232</v>
@@ -3558,10 +3687,10 @@
         <v>240</v>
       </c>
       <c r="I27" t="s" s="0">
-        <v>549</v>
+        <v>558</v>
       </c>
       <c r="J27" t="s">
-        <v>550</v>
+        <v>559</v>
       </c>
       <c r="K27" t="s">
         <v>232</v>
@@ -3606,10 +3735,10 @@
         <v>241</v>
       </c>
       <c r="I28" t="s" s="0">
-        <v>551</v>
+        <v>560</v>
       </c>
       <c r="J28" t="s">
-        <v>552</v>
+        <v>561</v>
       </c>
       <c r="K28" t="s">
         <v>232</v>
@@ -3651,7 +3780,7 @@
         <v>488</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>510</v>
+        <v>562</v>
       </c>
       <c r="K29" t="s" s="0">
         <v>232</v>
@@ -3696,10 +3825,10 @@
         <v>242</v>
       </c>
       <c r="I30" t="s" s="0">
-        <v>553</v>
+        <v>563</v>
       </c>
       <c r="J30" t="s">
-        <v>554</v>
+        <v>564</v>
       </c>
       <c r="K30" t="s">
         <v>232</v>
@@ -3780,16 +3909,16 @@
         <v>97</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>555</v>
+        <v>565</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>451</v>
+        <v>566</v>
       </c>
       <c r="I32" t="s" s="0">
-        <v>556</v>
+        <v>567</v>
       </c>
       <c r="J32" t="s">
-        <v>557</v>
+        <v>568</v>
       </c>
       <c r="K32" t="s">
         <v>232</v>
@@ -3855,10 +3984,10 @@
         <v>243</v>
       </c>
       <c r="I36" t="s" s="0">
-        <v>558</v>
+        <v>569</v>
       </c>
       <c r="J36" t="s">
-        <v>559</v>
+        <v>570</v>
       </c>
       <c r="K36" t="s">
         <v>232</v>
@@ -3903,10 +4032,10 @@
         <v>244</v>
       </c>
       <c r="I37" t="s" s="0">
-        <v>560</v>
+        <v>571</v>
       </c>
       <c r="J37" t="s">
-        <v>561</v>
+        <v>572</v>
       </c>
       <c r="K37" t="s">
         <v>232</v>
@@ -3945,16 +4074,16 @@
         <v>109</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>562</v>
+        <v>573</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>245</v>
       </c>
       <c r="I38" t="s" s="0">
-        <v>563</v>
+        <v>574</v>
       </c>
       <c r="J38" t="s">
-        <v>564</v>
+        <v>575</v>
       </c>
       <c r="K38" t="s">
         <v>232</v>
@@ -4041,10 +4170,10 @@
         <v>246</v>
       </c>
       <c r="I40" t="s" s="0">
-        <v>565</v>
+        <v>576</v>
       </c>
       <c r="J40" t="s">
-        <v>566</v>
+        <v>577</v>
       </c>
       <c r="K40" t="s">
         <v>232</v>
@@ -4089,10 +4218,10 @@
         <v>247</v>
       </c>
       <c r="I41" t="s" s="0">
-        <v>567</v>
+        <v>578</v>
       </c>
       <c r="J41" t="s">
-        <v>568</v>
+        <v>579</v>
       </c>
       <c r="K41" t="s">
         <v>232</v>
@@ -4134,13 +4263,13 @@
         <v>442</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>511</v>
+        <v>580</v>
       </c>
       <c r="I42" t="s" s="0">
-        <v>569</v>
+        <v>581</v>
       </c>
       <c r="J42" t="s">
-        <v>570</v>
+        <v>582</v>
       </c>
       <c r="K42" t="s">
         <v>232</v>
@@ -4185,10 +4314,10 @@
         <v>248</v>
       </c>
       <c r="I43" t="s" s="0">
-        <v>571</v>
+        <v>583</v>
       </c>
       <c r="J43" t="s">
-        <v>572</v>
+        <v>584</v>
       </c>
       <c r="K43" t="s">
         <v>232</v>
@@ -4227,7 +4356,7 @@
         <v>142</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>562</v>
+        <v>573</v>
       </c>
       <c r="H44" s="3" t="s">
         <v>249</v>
@@ -4275,10 +4404,10 @@
         <v>250</v>
       </c>
       <c r="I45" t="s" s="0">
-        <v>573</v>
+        <v>585</v>
       </c>
       <c r="J45" t="s">
-        <v>574</v>
+        <v>586</v>
       </c>
       <c r="K45" t="s">
         <v>232</v>
@@ -4323,10 +4452,10 @@
         <v>453</v>
       </c>
       <c r="I46" t="s" s="0">
-        <v>575</v>
+        <v>587</v>
       </c>
       <c r="J46" t="s">
-        <v>576</v>
+        <v>588</v>
       </c>
       <c r="K46" t="s">
         <v>232</v>
@@ -4368,13 +4497,13 @@
         <v>186</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>511</v>
+        <v>580</v>
       </c>
       <c r="I47" t="s" s="0">
-        <v>577</v>
+        <v>589</v>
       </c>
       <c r="J47" t="s">
-        <v>578</v>
+        <v>590</v>
       </c>
       <c r="K47" t="s">
         <v>232</v>
@@ -4419,10 +4548,10 @@
         <v>239</v>
       </c>
       <c r="I48" t="s" s="0">
-        <v>579</v>
+        <v>591</v>
       </c>
       <c r="J48" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="K48" t="s">
         <v>232</v>
@@ -4467,10 +4596,10 @@
         <v>251</v>
       </c>
       <c r="I49" t="s" s="0">
-        <v>581</v>
+        <v>593</v>
       </c>
       <c r="J49" t="s">
-        <v>582</v>
+        <v>594</v>
       </c>
       <c r="K49" t="s">
         <v>232</v>
@@ -4509,7 +4638,7 @@
         <v>146</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>562</v>
+        <v>573</v>
       </c>
       <c r="H50" s="3" t="s">
         <v>252</v>
@@ -4557,10 +4686,10 @@
         <v>253</v>
       </c>
       <c r="I51" t="s" s="0">
-        <v>583</v>
+        <v>595</v>
       </c>
       <c r="J51" t="s">
-        <v>584</v>
+        <v>596</v>
       </c>
       <c r="K51" t="s">
         <v>232</v>
@@ -4602,13 +4731,13 @@
         <v>190</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>454</v>
+        <v>597</v>
       </c>
       <c r="I52" t="s" s="0">
-        <v>585</v>
+        <v>598</v>
       </c>
       <c r="J52" t="s">
-        <v>586</v>
+        <v>599</v>
       </c>
       <c r="K52" t="s">
         <v>232</v>
@@ -4650,13 +4779,13 @@
         <v>191</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>462</v>
+        <v>600</v>
       </c>
       <c r="I53" t="s" s="0">
-        <v>587</v>
+        <v>601</v>
       </c>
       <c r="J53" t="s">
-        <v>588</v>
+        <v>602</v>
       </c>
       <c r="K53" t="s">
         <v>232</v>
@@ -4740,13 +4869,13 @@
         <v>193</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>455</v>
+        <v>603</v>
       </c>
       <c r="I55" t="s" s="0">
-        <v>589</v>
+        <v>604</v>
       </c>
       <c r="J55" t="s">
-        <v>590</v>
+        <v>605</v>
       </c>
       <c r="K55" t="s">
         <v>232</v>
@@ -4812,7 +4941,7 @@
         <v>491</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>463</v>
+        <v>606</v>
       </c>
       <c r="K60" t="s" s="0">
         <v>232</v>
@@ -4896,13 +5025,13 @@
         <v>194</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>464</v>
+        <v>607</v>
       </c>
       <c r="I62" t="s" s="0">
-        <v>591</v>
+        <v>608</v>
       </c>
       <c r="J62" t="s">
-        <v>592</v>
+        <v>609</v>
       </c>
       <c r="K62" t="s">
         <v>232</v>
@@ -4986,10 +5115,10 @@
         <v>256</v>
       </c>
       <c r="I64" t="s" s="0">
-        <v>593</v>
+        <v>610</v>
       </c>
       <c r="J64" t="s">
-        <v>594</v>
+        <v>611</v>
       </c>
       <c r="K64" t="s">
         <v>232</v>
@@ -5031,10 +5160,10 @@
         <v>257</v>
       </c>
       <c r="I65" t="s" s="0">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="J65" t="s">
-        <v>596</v>
+        <v>613</v>
       </c>
       <c r="K65" t="s">
         <v>232</v>
@@ -5073,13 +5202,13 @@
         <v>198</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>465</v>
+        <v>614</v>
       </c>
       <c r="I66" t="s" s="0">
-        <v>597</v>
+        <v>615</v>
       </c>
       <c r="J66" t="s">
-        <v>598</v>
+        <v>616</v>
       </c>
       <c r="K66" t="s">
         <v>232</v>
@@ -5166,10 +5295,10 @@
         <v>259</v>
       </c>
       <c r="I68" t="s" s="0">
-        <v>599</v>
+        <v>617</v>
       </c>
       <c r="J68" t="s">
-        <v>600</v>
+        <v>618</v>
       </c>
       <c r="K68" t="s">
         <v>232</v>
@@ -5214,10 +5343,10 @@
         <v>260</v>
       </c>
       <c r="I69" t="s" s="0">
-        <v>601</v>
+        <v>619</v>
       </c>
       <c r="J69" t="s">
-        <v>602</v>
+        <v>620</v>
       </c>
       <c r="K69" t="s">
         <v>232</v>
@@ -5262,10 +5391,10 @@
         <v>456</v>
       </c>
       <c r="I70" t="s" s="0">
-        <v>603</v>
+        <v>621</v>
       </c>
       <c r="J70" t="s">
-        <v>604</v>
+        <v>622</v>
       </c>
       <c r="K70" t="s">
         <v>232</v>
@@ -5307,13 +5436,13 @@
         <v>202</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>466</v>
+        <v>623</v>
       </c>
       <c r="I71" t="s" s="0">
-        <v>605</v>
+        <v>624</v>
       </c>
       <c r="J71" t="s">
-        <v>606</v>
+        <v>625</v>
       </c>
       <c r="K71" t="s">
         <v>232</v>
@@ -5397,13 +5526,13 @@
         <v>203</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>467</v>
+        <v>626</v>
       </c>
       <c r="I73" t="s" s="0">
-        <v>607</v>
+        <v>627</v>
       </c>
       <c r="J73" t="s">
-        <v>608</v>
+        <v>628</v>
       </c>
       <c r="K73" t="s">
         <v>232</v>
@@ -5448,10 +5577,10 @@
         <v>262</v>
       </c>
       <c r="I74" t="s" s="0">
-        <v>609</v>
+        <v>629</v>
       </c>
       <c r="J74" t="s">
-        <v>610</v>
+        <v>630</v>
       </c>
       <c r="K74" t="s">
         <v>232</v>
@@ -5493,13 +5622,13 @@
         <v>205</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>457</v>
+        <v>631</v>
       </c>
       <c r="I75" t="s" s="0">
-        <v>611</v>
+        <v>632</v>
       </c>
       <c r="J75" t="s">
-        <v>612</v>
+        <v>633</v>
       </c>
       <c r="K75" t="s">
         <v>232</v>
@@ -5538,16 +5667,16 @@
         <v>152</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>613</v>
+        <v>634</v>
       </c>
       <c r="H76" s="3" t="s">
         <v>263</v>
       </c>
       <c r="I76" t="s" s="0">
-        <v>614</v>
+        <v>635</v>
       </c>
       <c r="J76" t="s">
-        <v>615</v>
+        <v>636</v>
       </c>
       <c r="K76" t="s">
         <v>232</v>
@@ -5586,16 +5715,16 @@
         <v>153</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>616</v>
+        <v>637</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>468</v>
+        <v>638</v>
       </c>
       <c r="I77" t="s" s="0">
-        <v>617</v>
+        <v>639</v>
       </c>
       <c r="J77" t="s">
-        <v>618</v>
+        <v>640</v>
       </c>
       <c r="K77" t="s">
         <v>232</v>
@@ -5643,13 +5772,13 @@
         <v>206</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>458</v>
+        <v>641</v>
       </c>
       <c r="I79" t="s" s="0">
-        <v>619</v>
+        <v>642</v>
       </c>
       <c r="J79" t="s">
-        <v>620</v>
+        <v>643</v>
       </c>
       <c r="K79" t="s">
         <v>232</v>
@@ -5691,13 +5820,13 @@
         <v>207</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>469</v>
+        <v>644</v>
       </c>
       <c r="I80" t="s" s="0">
-        <v>621</v>
+        <v>645</v>
       </c>
       <c r="J80" t="s">
-        <v>622</v>
+        <v>646</v>
       </c>
       <c r="K80" t="s">
         <v>232</v>
@@ -5742,10 +5871,10 @@
         <v>264</v>
       </c>
       <c r="I81" t="s" s="0">
-        <v>623</v>
+        <v>647</v>
       </c>
       <c r="J81" t="s">
-        <v>624</v>
+        <v>648</v>
       </c>
       <c r="K81" t="s">
         <v>232</v>
@@ -5787,13 +5916,13 @@
         <v>209</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>470</v>
+        <v>649</v>
       </c>
       <c r="I82" t="s" s="0">
-        <v>625</v>
+        <v>650</v>
       </c>
       <c r="J82" t="s">
-        <v>626</v>
+        <v>651</v>
       </c>
       <c r="K82" t="s">
         <v>232</v>
@@ -5835,7 +5964,7 @@
         <v>210</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>459</v>
+        <v>652</v>
       </c>
       <c r="K83" t="s" s="0">
         <v>232</v>
@@ -5877,10 +6006,10 @@
         <v>265</v>
       </c>
       <c r="I84" t="s" s="0">
-        <v>627</v>
+        <v>653</v>
       </c>
       <c r="J84" t="s">
-        <v>628</v>
+        <v>654</v>
       </c>
       <c r="K84" t="s">
         <v>232</v>
@@ -5932,10 +6061,10 @@
         <v>266</v>
       </c>
       <c r="I86" t="s" s="0">
-        <v>629</v>
+        <v>655</v>
       </c>
       <c r="J86" t="s">
-        <v>630</v>
+        <v>656</v>
       </c>
       <c r="K86" t="s">
         <v>232</v>
@@ -5980,10 +6109,10 @@
         <v>267</v>
       </c>
       <c r="I87" t="s" s="0">
-        <v>631</v>
+        <v>657</v>
       </c>
       <c r="J87" t="s">
-        <v>632</v>
+        <v>658</v>
       </c>
       <c r="K87" t="s">
         <v>232</v>
@@ -6025,13 +6154,13 @@
         <v>214</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>471</v>
+        <v>659</v>
       </c>
       <c r="I88" t="s" s="0">
-        <v>633</v>
+        <v>660</v>
       </c>
       <c r="J88" t="s">
-        <v>634</v>
+        <v>661</v>
       </c>
       <c r="K88" t="s">
         <v>232</v>
@@ -6073,13 +6202,13 @@
         <v>215</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>495</v>
+        <v>662</v>
       </c>
       <c r="I89" t="s" s="0">
-        <v>635</v>
+        <v>663</v>
       </c>
       <c r="J89" t="s">
-        <v>636</v>
+        <v>664</v>
       </c>
       <c r="K89" t="s">
         <v>232</v>
@@ -6163,10 +6292,10 @@
         <v>269</v>
       </c>
       <c r="I91" t="s" s="0">
-        <v>637</v>
+        <v>665</v>
       </c>
       <c r="J91" t="s">
-        <v>638</v>
+        <v>666</v>
       </c>
       <c r="K91" t="s">
         <v>232</v>
@@ -6208,13 +6337,13 @@
         <v>217</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>472</v>
+        <v>667</v>
       </c>
       <c r="I92" t="s" s="0">
-        <v>639</v>
+        <v>668</v>
       </c>
       <c r="J92" t="s">
-        <v>640</v>
+        <v>669</v>
       </c>
       <c r="K92" t="s">
         <v>232</v>
@@ -6257,13 +6386,13 @@
         <v>218</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>496</v>
+        <v>670</v>
       </c>
       <c r="I93" t="s" s="0">
-        <v>641</v>
+        <v>671</v>
       </c>
       <c r="J93" t="s">
-        <v>642</v>
+        <v>672</v>
       </c>
       <c r="K93" t="s">
         <v>232</v>
@@ -6303,7 +6432,7 @@
       </c>
       <c r="G94" s="1"/>
       <c r="H94" s="3" t="s">
-        <v>473</v>
+        <v>673</v>
       </c>
       <c r="K94" t="s" s="0">
         <v>232</v>
@@ -6348,10 +6477,10 @@
         <v>270</v>
       </c>
       <c r="I95" t="s" s="0">
-        <v>643</v>
+        <v>674</v>
       </c>
       <c r="J95" t="s">
-        <v>644</v>
+        <v>675</v>
       </c>
       <c r="K95" t="s">
         <v>232</v>
@@ -6435,13 +6564,13 @@
         <v>220</v>
       </c>
       <c r="H102" s="3" t="s">
-        <v>460</v>
+        <v>676</v>
       </c>
       <c r="I102" t="s" s="0">
-        <v>645</v>
+        <v>677</v>
       </c>
       <c r="J102" t="s">
-        <v>646</v>
+        <v>678</v>
       </c>
       <c r="K102" t="s">
         <v>232</v>
@@ -6486,10 +6615,10 @@
         <v>443</v>
       </c>
       <c r="I103" t="s" s="0">
-        <v>647</v>
+        <v>679</v>
       </c>
       <c r="J103" t="s">
-        <v>648</v>
+        <v>680</v>
       </c>
       <c r="K103" t="s">
         <v>232</v>
@@ -6534,10 +6663,10 @@
         <v>271</v>
       </c>
       <c r="I104" t="s" s="0">
-        <v>649</v>
+        <v>681</v>
       </c>
       <c r="J104" t="s">
-        <v>650</v>
+        <v>682</v>
       </c>
       <c r="K104" t="s">
         <v>232</v>
@@ -6621,13 +6750,13 @@
         <v>224</v>
       </c>
       <c r="H106" s="3" t="s">
-        <v>461</v>
+        <v>683</v>
       </c>
       <c r="I106" t="s" s="0">
-        <v>651</v>
+        <v>684</v>
       </c>
       <c r="J106" t="s">
-        <v>652</v>
+        <v>685</v>
       </c>
       <c r="K106" t="s">
         <v>232</v>
@@ -6809,7 +6938,7 @@
         <v>218</v>
       </c>
       <c r="H127" s="3" t="s">
-        <v>497</v>
+        <v>686</v>
       </c>
       <c r="K127" t="s" s="0">
         <v>232</v>
@@ -6851,13 +6980,13 @@
         <v>225</v>
       </c>
       <c r="H128" s="3" t="s">
-        <v>498</v>
+        <v>687</v>
       </c>
       <c r="I128" t="s" s="0">
-        <v>653</v>
+        <v>688</v>
       </c>
       <c r="J128" t="s">
-        <v>654</v>
+        <v>689</v>
       </c>
       <c r="K128" t="s">
         <v>232</v>
@@ -6899,13 +7028,13 @@
         <v>226</v>
       </c>
       <c r="H129" s="3" t="s">
-        <v>499</v>
+        <v>690</v>
       </c>
       <c r="I129" t="s" s="0">
-        <v>655</v>
+        <v>691</v>
       </c>
       <c r="J129" t="s">
-        <v>656</v>
+        <v>692</v>
       </c>
       <c r="K129" t="s">
         <v>232</v>
@@ -6947,7 +7076,7 @@
         <v>226</v>
       </c>
       <c r="H130" s="3" t="s">
-        <v>500</v>
+        <v>693</v>
       </c>
       <c r="K130" t="s" s="0">
         <v>232</v>
@@ -6989,13 +7118,13 @@
         <v>227</v>
       </c>
       <c r="H131" s="3" t="s">
-        <v>501</v>
+        <v>694</v>
       </c>
       <c r="I131" t="s" s="0">
-        <v>657</v>
+        <v>695</v>
       </c>
       <c r="J131" t="s">
-        <v>658</v>
+        <v>696</v>
       </c>
       <c r="K131" t="s">
         <v>232</v>
@@ -7037,13 +7166,13 @@
         <v>228</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>502</v>
+        <v>697</v>
       </c>
       <c r="I132" t="s" s="0">
-        <v>659</v>
+        <v>698</v>
       </c>
       <c r="J132" t="s">
-        <v>660</v>
+        <v>699</v>
       </c>
       <c r="K132" t="s">
         <v>400</v>
@@ -7085,13 +7214,13 @@
         <v>229</v>
       </c>
       <c r="H133" s="3" t="s">
-        <v>503</v>
+        <v>700</v>
       </c>
       <c r="I133" t="s" s="0">
-        <v>661</v>
+        <v>701</v>
       </c>
       <c r="J133" t="s">
-        <v>662</v>
+        <v>702</v>
       </c>
       <c r="K133" t="s">
         <v>232</v>
@@ -7133,13 +7262,13 @@
         <v>230</v>
       </c>
       <c r="H134" s="3" t="s">
-        <v>504</v>
+        <v>703</v>
       </c>
       <c r="I134" t="s" s="0">
-        <v>663</v>
+        <v>704</v>
       </c>
       <c r="J134" t="s">
-        <v>664</v>
+        <v>705</v>
       </c>
       <c r="K134" t="s">
         <v>232</v>
@@ -7179,7 +7308,7 @@
       </c>
       <c r="G135" s="1"/>
       <c r="H135" s="3" t="s">
-        <v>505</v>
+        <v>706</v>
       </c>
       <c r="K135" t="s" s="0">
         <v>232</v>
@@ -7221,13 +7350,13 @@
         <v>231</v>
       </c>
       <c r="H136" s="3" t="s">
-        <v>506</v>
+        <v>707</v>
       </c>
       <c r="I136" t="s" s="0">
-        <v>665</v>
+        <v>708</v>
       </c>
       <c r="J136" t="s">
-        <v>666</v>
+        <v>709</v>
       </c>
       <c r="K136" t="s">
         <v>232</v>

</xml_diff>